<commit_message>
changed to mac and added the evaluations as well as metrics
</commit_message>
<xml_diff>
--- a/data/ground_truth_evals/product_info.xlsx
+++ b/data/ground_truth_evals/product_info.xlsx
@@ -265,6 +265,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
fixed some changes on the truth values of the evals and turned the AI Orchestrator into a class to avoid remaking the chain on every function call
</commit_message>
<xml_diff>
--- a/data/ground_truth_evals/product_info.xlsx
+++ b/data/ground_truth_evals/product_info.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://upvedues-my.sharepoint.com/personal/gmarpea_upv_edu_es/Documents/SYNC/Code/Projects/Mercadona-LLM/data/ground_truth_evals/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\code\projects\AI-Product-Recommender\data\ground_truth_evals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{1D33A2DE-F877-4B09-9861-CDACDDFC2F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65890050-5510-4663-B272-D6D8170FA518}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC79668-3D63-4578-9F54-E749D081316F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB5ABBB8-4630-4D24-9149-74D7A2322810}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="60">
   <si>
     <t>ID_producto</t>
   </si>
@@ -92,18 +92,12 @@
     <t>sin azucar anadido</t>
   </si>
   <si>
-    <t>cereales, gluten, lactosa, frutos de cascara, soja</t>
-  </si>
-  <si>
     <t>Kellogg's</t>
   </si>
   <si>
     <t>caro</t>
   </si>
   <si>
-    <t>cereales, gluten</t>
-  </si>
-  <si>
     <t>Campo Nature</t>
   </si>
   <si>
@@ -122,18 +116,12 @@
     <t>fuente de fibra</t>
   </si>
   <si>
-    <t>Enervit Sport</t>
-  </si>
-  <si>
     <t>lactosa, soja, frutos de cascara, sesamo, cacahuete</t>
   </si>
   <si>
     <t>alto en proteina, bajo en azucar</t>
   </si>
   <si>
-    <t>standard</t>
-  </si>
-  <si>
     <t>cereal, gluten, lactosa, soja, mostaza</t>
   </si>
   <si>
@@ -155,27 +143,12 @@
     <t>pescado</t>
   </si>
   <si>
-    <t>marisco, moluscos, pescado</t>
-  </si>
-  <si>
-    <t>cereal, gluten, lactosa, sesamo, frutos de cascara, soja, sulfitos, moluscos, pescado, mostaza, cacahuetes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">standard </t>
-  </si>
-  <si>
     <t>gluten, lactosa, soja, sesamo, mostaza</t>
   </si>
   <si>
     <t>lactosa</t>
   </si>
   <si>
-    <t>bajo en azucar</t>
-  </si>
-  <si>
-    <t>bajo en azucar, alto en proteina</t>
-  </si>
-  <si>
     <t>muy barato</t>
   </si>
   <si>
@@ -206,13 +179,43 @@
     <t>caro|muy caro</t>
   </si>
   <si>
-    <t>standard|caro</t>
-  </si>
-  <si>
     <t>barato|muy barato</t>
   </si>
   <si>
-    <t>standard|barato</t>
+    <t>cereal, gluten, lactosa, frutos de cascara, soja</t>
+  </si>
+  <si>
+    <t>cereal, gluten</t>
+  </si>
+  <si>
+    <t>cereal, gluten, lactosa, sesamo, frutos de cascara, soja, sulfitos, moluscos, pescado, mostaza, cacahuete</t>
+  </si>
+  <si>
+    <t>Enervit</t>
+  </si>
+  <si>
+    <t>estandar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">estandar </t>
+  </si>
+  <si>
+    <t>estandar|barato</t>
+  </si>
+  <si>
+    <t>estandar|caro</t>
+  </si>
+  <si>
+    <t>marisco, moluscos, pescado, sulfitos</t>
+  </si>
+  <si>
+    <t>bajo en azucar, bajo en grasa</t>
+  </si>
+  <si>
+    <t>bajo en grasa, alto en proteina</t>
+  </si>
+  <si>
+    <t>sulfitos, cereal</t>
   </si>
 </sst>
 </file>
@@ -265,10 +268,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -658,7 +657,7 @@
         <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -696,13 +695,13 @@
         <v>9210</v>
       </c>
       <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="F3">
         <v>1604</v>
@@ -740,7 +739,7 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="F4">
         <v>3378</v>
@@ -775,13 +774,13 @@
         <v>21756</v>
       </c>
       <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
         <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
       </c>
       <c r="F5">
         <v>1502</v>
@@ -816,16 +815,16 @@
         <v>19958</v>
       </c>
       <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
         <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" t="s">
-        <v>27</v>
       </c>
       <c r="F6">
         <v>79</v>
@@ -860,16 +859,16 @@
         <v>19867</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F7">
         <v>1612</v>
@@ -907,13 +906,13 @@
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F8">
         <v>1996</v>
@@ -931,7 +930,7 @@
         <v>61</v>
       </c>
       <c r="K8">
-        <v>1.8</v>
+        <v>18</v>
       </c>
       <c r="L8">
         <v>6.8</v>
@@ -954,7 +953,7 @@
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F9">
         <v>2068</v>
@@ -989,16 +988,16 @@
         <v>14269</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F10">
         <v>512</v>
@@ -1036,10 +1035,10 @@
         <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F11">
         <v>1155</v>
@@ -1077,10 +1076,10 @@
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F12">
         <v>1371</v>
@@ -1118,10 +1117,10 @@
         <v>14</v>
       </c>
       <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" t="s">
         <v>56</v>
-      </c>
-      <c r="D13" t="s">
-        <v>39</v>
       </c>
       <c r="F13">
         <v>326</v>
@@ -1162,7 +1161,7 @@
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F14">
         <v>2097</v>
@@ -1200,10 +1199,10 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F15">
         <v>1121</v>
@@ -1243,8 +1242,11 @@
       <c r="C16" t="s">
         <v>15</v>
       </c>
+      <c r="D16" t="s">
+        <v>36</v>
+      </c>
       <c r="E16" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="F16">
         <v>204</v>
@@ -1285,16 +1287,16 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E17" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="F17">
         <v>226</v>
       </c>
       <c r="G17">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H17">
         <v>0.5</v>
@@ -1326,7 +1328,7 @@
         <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="F18">
         <v>1462</v>
@@ -1361,16 +1363,16 @@
         <v>13926</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="D19" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E19" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F19">
         <v>1517</v>
@@ -1408,7 +1410,10 @@
         <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>47</v>
+      </c>
+      <c r="D20" t="s">
+        <v>42</v>
       </c>
       <c r="F20">
         <v>350</v>
@@ -1443,13 +1448,13 @@
         <v>13204</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C21" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D21" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="F21">
         <v>1634</v>
@@ -1487,10 +1492,10 @@
         <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="F22">
         <v>905</v>
@@ -1525,13 +1530,13 @@
         <v>12562</v>
       </c>
       <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
         <v>52</v>
       </c>
-      <c r="C23" t="s">
-        <v>31</v>
-      </c>
       <c r="D23" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="F23">
         <v>2248</v>
@@ -1569,7 +1574,7 @@
         <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="F24">
         <v>833</v>
@@ -1604,13 +1609,13 @@
         <v>10502</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="D25" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F25">
         <v>194</v>

</xml_diff>

<commit_message>
fixed bugs and completed eval implementation
</commit_message>
<xml_diff>
--- a/data/ground_truth_evals/product_info.xlsx
+++ b/data/ground_truth_evals/product_info.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\code\projects\AI-Product-Recommender\data\ground_truth_evals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC79668-3D63-4578-9F54-E749D081316F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28598B2-1840-48FC-8451-7C7101AFD19F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB5ABBB8-4630-4D24-9149-74D7A2322810}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
   <si>
     <t>ID_producto</t>
   </si>
@@ -110,9 +110,6 @@
     <t>Antonio</t>
   </si>
   <si>
-    <t>mostaza, sesamo</t>
-  </si>
-  <si>
     <t>fuente de fibra</t>
   </si>
   <si>
@@ -122,12 +119,6 @@
     <t>alto en proteina, bajo en azucar</t>
   </si>
   <si>
-    <t>cereal, gluten, lactosa, soja, mostaza</t>
-  </si>
-  <si>
-    <t>cereal, gluten, lactosa, mostaza, frutos de cascara, huevo, soja</t>
-  </si>
-  <si>
     <t>La Carloteña</t>
   </si>
   <si>
@@ -158,9 +149,6 @@
     <t>soja</t>
   </si>
   <si>
-    <t>fuente de fibra, vegetariano, bajo en grasa, alto en proteina</t>
-  </si>
-  <si>
     <t>Nesquik</t>
   </si>
   <si>
@@ -182,15 +170,6 @@
     <t>barato|muy barato</t>
   </si>
   <si>
-    <t>cereal, gluten, lactosa, frutos de cascara, soja</t>
-  </si>
-  <si>
-    <t>cereal, gluten</t>
-  </si>
-  <si>
-    <t>cereal, gluten, lactosa, sesamo, frutos de cascara, soja, sulfitos, moluscos, pescado, mostaza, cacahuete</t>
-  </si>
-  <si>
     <t>Enervit</t>
   </si>
   <si>
@@ -215,7 +194,25 @@
     <t>bajo en grasa, alto en proteina</t>
   </si>
   <si>
-    <t>sulfitos, cereal</t>
+    <t>gluten, lactosa, frutos de cascara, soja</t>
+  </si>
+  <si>
+    <t>gluten</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> gluten, lactosa, soja, mostaza</t>
+  </si>
+  <si>
+    <t>gluten, lactosa, mostaza, frutos de cascara, huevo, soja</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> gluten, lactosa, sesamo, frutos de cascara, soja, sulfitos, moluscos, pescado, mostaza, cacahuete</t>
+  </si>
+  <si>
+    <t>mostaza, sesamo, sulfitos</t>
+  </si>
+  <si>
+    <t>fuente de fibra, vegetariano, bajo en grasa, alto en proteina, vegano</t>
   </si>
 </sst>
 </file>
@@ -657,7 +654,7 @@
         <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -701,7 +698,7 @@
         <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F3">
         <v>1604</v>
@@ -739,7 +736,7 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F4">
         <v>3378</v>
@@ -818,13 +815,13 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E6" t="s">
         <v>24</v>
-      </c>
-      <c r="E6" t="s">
-        <v>25</v>
       </c>
       <c r="F6">
         <v>79</v>
@@ -859,16 +856,16 @@
         <v>19867</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
         <v>21</v>
       </c>
       <c r="D7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" t="s">
         <v>26</v>
-      </c>
-      <c r="E7" t="s">
-        <v>27</v>
       </c>
       <c r="F7">
         <v>1612</v>
@@ -906,13 +903,13 @@
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F8">
         <v>1996</v>
@@ -953,7 +950,7 @@
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="F9">
         <v>2068</v>
@@ -988,16 +985,16 @@
         <v>14269</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F10">
         <v>512</v>
@@ -1035,10 +1032,10 @@
         <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F11">
         <v>1155</v>
@@ -1076,10 +1073,10 @@
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F12">
         <v>1371</v>
@@ -1117,10 +1114,10 @@
         <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="F13">
         <v>326</v>
@@ -1155,13 +1152,13 @@
         <v>84629</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C14" t="s">
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F14">
         <v>2097</v>
@@ -1196,13 +1193,13 @@
         <v>14431</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F15">
         <v>1121</v>
@@ -1243,10 +1240,10 @@
         <v>15</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="F16">
         <v>204</v>
@@ -1287,10 +1284,10 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E17" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="F17">
         <v>226</v>
@@ -1328,7 +1325,7 @@
         <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F18">
         <v>1462</v>
@@ -1363,16 +1360,16 @@
         <v>13926</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D19" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E19" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="F19">
         <v>1517</v>
@@ -1410,10 +1407,10 @@
         <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F20">
         <v>350</v>
@@ -1448,13 +1445,13 @@
         <v>13204</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D21" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F21">
         <v>1634</v>
@@ -1489,13 +1486,13 @@
         <v>52672</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D22" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="F22">
         <v>905</v>
@@ -1530,13 +1527,13 @@
         <v>12562</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D23" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F23">
         <v>2248</v>
@@ -1574,7 +1571,7 @@
         <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F24">
         <v>833</v>
@@ -1609,13 +1606,13 @@
         <v>10502</v>
       </c>
       <c r="B25" t="s">
+        <v>41</v>
+      </c>
+      <c r="C25" t="s">
         <v>45</v>
       </c>
-      <c r="C25" t="s">
-        <v>52</v>
-      </c>
       <c r="D25" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F25">
         <v>194</v>

</xml_diff>

<commit_message>
updated errors and implemented reflection for allergens
</commit_message>
<xml_diff>
--- a/data/ground_truth_evals/product_info.xlsx
+++ b/data/ground_truth_evals/product_info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\code\projects\AI-Product-Recommender\data\ground_truth_evals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28598B2-1840-48FC-8451-7C7101AFD19F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B3A74A-034E-482A-B933-35082BC4145C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB5ABBB8-4630-4D24-9149-74D7A2322810}"/>
   </bookViews>
@@ -206,13 +206,13 @@
     <t>gluten, lactosa, mostaza, frutos de cascara, huevo, soja</t>
   </si>
   <si>
-    <t xml:space="preserve"> gluten, lactosa, sesamo, frutos de cascara, soja, sulfitos, moluscos, pescado, mostaza, cacahuete</t>
-  </si>
-  <si>
     <t>mostaza, sesamo, sulfitos</t>
   </si>
   <si>
     <t>fuente de fibra, vegetariano, bajo en grasa, alto en proteina, vegano</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> gluten, lactosa, sesamo, frutos de cascara, soja, sulfitos, moluscos, pescado, mostaza, cacahuete, huevo</t>
   </si>
 </sst>
 </file>
@@ -818,7 +818,7 @@
         <v>42</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E6" t="s">
         <v>24</v>
@@ -1158,7 +1158,7 @@
         <v>15</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F14">
         <v>2097</v>
@@ -1369,7 +1369,7 @@
         <v>36</v>
       </c>
       <c r="E19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F19">
         <v>1517</v>

</xml_diff>